<commit_message>
Ajustes da Cãmera pra poder ser usada
</commit_message>
<xml_diff>
--- a/modelos/modelo de faturamento.xlsx
+++ b/modelos/modelo de faturamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AEEEB0D4-5546-40E5-BF56-3B8C73DCAA02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{AEEEB0D4-5546-40E5-BF56-3B8C73DCAA02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63B79E6C-B285-4E14-A686-E115FF0448B6}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{231199EE-4300-4F8B-A0B3-A2B2F5200136}"/>
   </bookViews>
@@ -19,6 +19,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">Planilha1!$A$1:$F$14</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -200,7 +201,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -226,15 +227,6 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -245,7 +237,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -259,29 +251,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -347,10 +333,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -681,7 +663,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="29.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8"/>
+      <c r="A1" s="9"/>
       <c r="B1" s="10" t="s">
         <v>4</v>
       </c>
@@ -692,132 +674,132 @@
     </row>
     <row r="2" spans="1:11" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
     </row>
     <row r="3" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
     </row>
     <row r="4" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
     </row>
     <row r="5" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
     </row>
     <row r="6" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
     </row>
     <row r="7" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
     </row>
     <row r="8" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
     </row>
     <row r="9" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
     </row>
     <row r="10" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
     </row>
     <row r="11" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
       <c r="K13" s="4"/>
     </row>
     <row r="14" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A15" s="5"/>
@@ -856,6 +838,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="A1:A2"/>
@@ -864,12 +852,6 @@
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B1:F2"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.47" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" scale="63" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>